<commit_message>
breif save button added
</commit_message>
<xml_diff>
--- a/storage/app/Colombo_brief_upload.xlsx
+++ b/storage/app/Colombo_brief_upload.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="15">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="17">
   <si>
     <t>#</t>
   </si>
@@ -48,6 +48,12 @@
   </si>
   <si>
     <t>2025/04/11</t>
+  </si>
+  <si>
+    <t>ABC</t>
+  </si>
+  <si>
+    <t>Sri Lanka</t>
   </si>
   <si>
     <t>colombo5</t>
@@ -451,16 +457,24 @@
       <c r="C2">
         <v>5</v>
       </c>
-      <c r="D2"/>
-      <c r="E2"/>
-      <c r="F2"/>
-      <c r="G2"/>
+      <c r="D2" t="s">
+        <v>11</v>
+      </c>
+      <c r="E2" t="s">
+        <v>12</v>
+      </c>
+      <c r="F2">
+        <v>5</v>
+      </c>
+      <c r="G2">
+        <v>10</v>
+      </c>
       <c r="H2" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="I2"/>
       <c r="J2" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="K2"/>
       <c r="L2"/>
@@ -492,7 +506,7 @@
       <c r="H3"/>
       <c r="I3"/>
       <c r="J3" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="K3"/>
       <c r="L3"/>
@@ -524,7 +538,7 @@
       <c r="H4"/>
       <c r="I4"/>
       <c r="J4" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="K4"/>
       <c r="L4"/>

</xml_diff>

<commit_message>
project brief filter created
</commit_message>
<xml_diff>
--- a/storage/app/Colombo_brief_upload.xlsx
+++ b/storage/app/Colombo_brief_upload.xlsx
@@ -23,7 +23,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>Job Order No.</t>
+    <t>Job Order No</t>
   </si>
   <si>
     <t>Company Name</t>
@@ -38,7 +38,7 @@
     <t>Total CVs</t>
   </si>
   <si>
-    <t>Balancr Req No.</t>
+    <t>Balance Req No.</t>
   </si>
   <si>
     <t>Remark</t>

</xml_diff>